<commit_message>
supp tables for new papers
</commit_message>
<xml_diff>
--- a/data/Prochlorococcus/papers_and_supp/moreno 2023/spectrum.03275-22-s0003.xlsx
+++ b/data/Prochlorococcus/papers_and_supp/moreno 2023/spectrum.03275-22-s0003.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11113"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jose/Dropbox/2022 Integrated proteomic and metabolomic analysis of glucose utilization/Versión Microbiology Spectrum/R1/Supplementary tables/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Osnat\Documents\GitHub\multiomics_biocypher_kg\data\Prochlorococcus\papers_and_supp\moreno 2023\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9B953F8-CE7D-3845-9C80-F311847DAB6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63B81C90-74B1-40DD-B28A-A7F3D548D948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="36380" windowHeight="21100" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Alteromonas in WH8102 cultures" sheetId="1" r:id="rId1"/>
     <sheet name="Alteromonas in WH7803 cultures" sheetId="4" r:id="rId2"/>
     <sheet name="Alteromonas in BL107 cultures" sheetId="5" r:id="rId3"/>
     <sheet name="Alteromonas in SS120 cultures" sheetId="6" r:id="rId4"/>
-    <sheet name="Alteromonas in MED$ cultures" sheetId="7" r:id="rId5"/>
+    <sheet name="Alteromonas in MED4 cultures" sheetId="7" r:id="rId5"/>
   </sheets>
   <calcPr calcId="140001"/>
   <extLst>
@@ -1579,7 +1579,7 @@
     <numFmt numFmtId="171" formatCode="0.0000"/>
     <numFmt numFmtId="172" formatCode="0.000"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
@@ -1713,46 +1713,46 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="42">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="171" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1761,43 +1761,43 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="172" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="172" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1824,24 +1824,24 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="11" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="11" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Bueno" xfId="1" builtinId="26"/>
+    <cellStyle name="Good" xfId="1" builtinId="26"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="1">
@@ -3012,63 +3012,63 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:BE189"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.33203125" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="8.28515625" defaultRowHeight="20.100000000000001" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="12.1640625" style="13" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="13.6640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="91.33203125" style="2" customWidth="1"/>
-    <col min="6" max="7" width="32.33203125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="33.1640625" style="2" customWidth="1"/>
-    <col min="9" max="10" width="32.33203125" style="2" customWidth="1"/>
-    <col min="11" max="11" width="33.1640625" style="2" customWidth="1"/>
-    <col min="12" max="13" width="32.33203125" style="2" customWidth="1"/>
-    <col min="14" max="14" width="33.1640625" style="2" customWidth="1"/>
-    <col min="15" max="15" width="32.33203125" style="2" customWidth="1"/>
-    <col min="16" max="17" width="33.1640625" style="2" customWidth="1"/>
-    <col min="18" max="18" width="32.33203125" style="2" customWidth="1"/>
-    <col min="19" max="20" width="33.1640625" style="2" customWidth="1"/>
-    <col min="21" max="21" width="32.33203125" style="2" customWidth="1"/>
-    <col min="22" max="23" width="33.1640625" style="2" customWidth="1"/>
-    <col min="24" max="24" width="11.6640625" style="2" customWidth="1"/>
-    <col min="25" max="25" width="10.6640625" style="2" customWidth="1"/>
-    <col min="26" max="26" width="10.33203125" style="2" customWidth="1"/>
-    <col min="27" max="27" width="13.1640625" style="2" customWidth="1"/>
-    <col min="28" max="28" width="13.83203125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" style="13" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="13.7109375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="91.28515625" style="2" customWidth="1"/>
+    <col min="6" max="7" width="32.28515625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="33.140625" style="2" customWidth="1"/>
+    <col min="9" max="10" width="32.28515625" style="2" customWidth="1"/>
+    <col min="11" max="11" width="33.140625" style="2" customWidth="1"/>
+    <col min="12" max="13" width="32.28515625" style="2" customWidth="1"/>
+    <col min="14" max="14" width="33.140625" style="2" customWidth="1"/>
+    <col min="15" max="15" width="32.28515625" style="2" customWidth="1"/>
+    <col min="16" max="17" width="33.140625" style="2" customWidth="1"/>
+    <col min="18" max="18" width="32.28515625" style="2" customWidth="1"/>
+    <col min="19" max="20" width="33.140625" style="2" customWidth="1"/>
+    <col min="21" max="21" width="32.28515625" style="2" customWidth="1"/>
+    <col min="22" max="23" width="33.140625" style="2" customWidth="1"/>
+    <col min="24" max="24" width="11.7109375" style="2" customWidth="1"/>
+    <col min="25" max="25" width="10.7109375" style="2" customWidth="1"/>
+    <col min="26" max="26" width="10.28515625" style="2" customWidth="1"/>
+    <col min="27" max="27" width="13.140625" style="2" customWidth="1"/>
+    <col min="28" max="28" width="13.85546875" style="2" customWidth="1"/>
     <col min="29" max="29" width="13" style="2" customWidth="1"/>
-    <col min="30" max="30" width="15.6640625" style="2" customWidth="1"/>
-    <col min="31" max="31" width="13.6640625" style="2" customWidth="1"/>
-    <col min="32" max="32" width="14.1640625" style="2" customWidth="1"/>
+    <col min="30" max="30" width="15.7109375" style="2" customWidth="1"/>
+    <col min="31" max="31" width="13.7109375" style="2" customWidth="1"/>
+    <col min="32" max="32" width="14.140625" style="2" customWidth="1"/>
     <col min="33" max="33" width="11" style="2" customWidth="1"/>
-    <col min="34" max="34" width="10.6640625" style="2" customWidth="1"/>
-    <col min="35" max="35" width="8.33203125" style="2"/>
-    <col min="36" max="36" width="13.1640625" style="2" customWidth="1"/>
+    <col min="34" max="34" width="10.7109375" style="2" customWidth="1"/>
+    <col min="35" max="35" width="8.28515625" style="2"/>
+    <col min="36" max="36" width="13.140625" style="2" customWidth="1"/>
     <col min="37" max="37" width="12" style="2" customWidth="1"/>
-    <col min="38" max="38" width="12.6640625" style="2" customWidth="1"/>
-    <col min="39" max="39" width="12.1640625" style="2" customWidth="1"/>
-    <col min="40" max="40" width="13.83203125" style="2" customWidth="1"/>
-    <col min="41" max="41" width="13.1640625" style="2" customWidth="1"/>
-    <col min="42" max="42" width="76.33203125" style="14" customWidth="1"/>
-    <col min="43" max="43" width="12.1640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="15.1640625" style="2" customWidth="1"/>
+    <col min="38" max="38" width="12.7109375" style="2" customWidth="1"/>
+    <col min="39" max="39" width="12.140625" style="2" customWidth="1"/>
+    <col min="40" max="40" width="13.85546875" style="2" customWidth="1"/>
+    <col min="41" max="41" width="13.140625" style="2" customWidth="1"/>
+    <col min="42" max="42" width="76.28515625" style="14" customWidth="1"/>
+    <col min="43" max="43" width="12.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="15.140625" style="2" customWidth="1"/>
     <col min="45" max="45" width="16" style="2" customWidth="1"/>
     <col min="46" max="46" width="10" style="2" customWidth="1"/>
-    <col min="47" max="47" width="14.83203125" style="2" customWidth="1"/>
-    <col min="48" max="48" width="12.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="14.85546875" style="2" customWidth="1"/>
+    <col min="48" max="48" width="12.140625" style="2" bestFit="1" customWidth="1"/>
     <col min="49" max="49" width="12" style="2" customWidth="1"/>
-    <col min="50" max="50" width="11.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="11.83203125" style="2" customWidth="1"/>
-    <col min="52" max="52" width="11.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="10.83203125" style="2" customWidth="1"/>
-    <col min="54" max="54" width="11.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="13.6640625" style="2" customWidth="1"/>
-    <col min="56" max="56" width="11.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="76.33203125" style="14" customWidth="1"/>
-    <col min="58" max="16384" width="8.33203125" style="2"/>
+    <col min="50" max="50" width="11.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="11.85546875" style="2" customWidth="1"/>
+    <col min="52" max="52" width="11.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="10.85546875" style="2" customWidth="1"/>
+    <col min="54" max="54" width="11.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="13.7109375" style="2" customWidth="1"/>
+    <col min="56" max="56" width="11.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="76.28515625" style="14" customWidth="1"/>
+    <col min="58" max="16384" width="8.28515625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:57" ht="32" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:57" ht="32.1" customHeight="1">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -3241,7 +3241,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="2" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A2" s="11" t="s">
         <v>226</v>
       </c>
@@ -3414,7 +3414,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="3" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A3" s="12" t="s">
         <v>126</v>
       </c>
@@ -3587,7 +3587,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="4" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A4" s="13" t="s">
         <v>286</v>
       </c>
@@ -3760,7 +3760,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="5" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A5" s="13" t="s">
         <v>284</v>
       </c>
@@ -3933,7 +3933,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="6" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A6" s="13" t="s">
         <v>348</v>
       </c>
@@ -4106,7 +4106,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="7" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A7" s="13" t="s">
         <v>212</v>
       </c>
@@ -4279,7 +4279,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="8" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A8" s="12" t="s">
         <v>144</v>
       </c>
@@ -4452,7 +4452,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="9" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A9" s="12" t="s">
         <v>17</v>
       </c>
@@ -4625,7 +4625,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A10" s="13" t="s">
         <v>346</v>
       </c>
@@ -4798,7 +4798,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="11" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A11" s="12" t="s">
         <v>39</v>
       </c>
@@ -4971,7 +4971,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>266</v>
       </c>
@@ -5144,7 +5144,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="13" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A13" s="12" t="s">
         <v>87</v>
       </c>
@@ -5317,7 +5317,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="14" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A14" s="12" t="s">
         <v>120</v>
       </c>
@@ -5490,7 +5490,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="15" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A15" s="12" t="s">
         <v>109</v>
       </c>
@@ -5663,7 +5663,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="16" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A16" s="12" t="s">
         <v>103</v>
       </c>
@@ -5836,7 +5836,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="17" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A17" s="12" t="s">
         <v>188</v>
       </c>
@@ -6009,7 +6009,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="18" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A18" s="13" t="s">
         <v>218</v>
       </c>
@@ -6182,7 +6182,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="19" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A19" s="13" t="s">
         <v>210</v>
       </c>
@@ -6355,7 +6355,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="20" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A20" s="12" t="s">
         <v>178</v>
       </c>
@@ -6528,7 +6528,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="21" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A21" s="11" t="s">
         <v>252</v>
       </c>
@@ -6701,7 +6701,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="22" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A22" s="12" t="s">
         <v>158</v>
       </c>
@@ -6874,7 +6874,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="23" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A23" s="11" t="s">
         <v>230</v>
       </c>
@@ -7047,7 +7047,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="24" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A24" s="13" t="s">
         <v>206</v>
       </c>
@@ -7220,7 +7220,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="25" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A25" s="11" t="s">
         <v>318</v>
       </c>
@@ -7393,7 +7393,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="26" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A26" s="13" t="s">
         <v>330</v>
       </c>
@@ -7566,7 +7566,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="27" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A27" s="13" t="s">
         <v>288</v>
       </c>
@@ -7739,7 +7739,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="28" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A28" s="13" t="s">
         <v>336</v>
       </c>
@@ -7912,7 +7912,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="29" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A29" s="12" t="s">
         <v>172</v>
       </c>
@@ -8085,7 +8085,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="30" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A30" s="11" t="s">
         <v>264</v>
       </c>
@@ -8258,7 +8258,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="31" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A31" s="11" t="s">
         <v>308</v>
       </c>
@@ -8431,7 +8431,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="32" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A32" s="13" t="s">
         <v>274</v>
       </c>
@@ -8604,7 +8604,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="33" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A33" s="11" t="s">
         <v>320</v>
       </c>
@@ -8777,7 +8777,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="34" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A34" s="12" t="s">
         <v>128</v>
       </c>
@@ -8950,7 +8950,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="35" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A35" s="12" t="s">
         <v>118</v>
       </c>
@@ -9123,7 +9123,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="36" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A36" s="11" t="s">
         <v>240</v>
       </c>
@@ -9296,7 +9296,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="37" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A37" s="11" t="s">
         <v>312</v>
       </c>
@@ -9469,7 +9469,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="38" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A38" s="11" t="s">
         <v>244</v>
       </c>
@@ -9642,7 +9642,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="39" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A39" s="12" t="s">
         <v>55</v>
       </c>
@@ -9815,7 +9815,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="40" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A40" s="11" t="s">
         <v>368</v>
       </c>
@@ -9988,7 +9988,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="41" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="41" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A41" s="13" t="s">
         <v>216</v>
       </c>
@@ -10161,7 +10161,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="42" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="42" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A42" s="12" t="s">
         <v>5</v>
       </c>
@@ -10334,7 +10334,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="43" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A43" s="11" t="s">
         <v>358</v>
       </c>
@@ -10507,7 +10507,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="44" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="44" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A44" s="12" t="s">
         <v>168</v>
       </c>
@@ -10680,7 +10680,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="45" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="45" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A45" s="13" t="s">
         <v>372</v>
       </c>
@@ -10853,7 +10853,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="46" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="46" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A46" s="13" t="s">
         <v>280</v>
       </c>
@@ -11026,7 +11026,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="47" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="47" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A47" s="13" t="s">
         <v>292</v>
       </c>
@@ -11199,7 +11199,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="48" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="48" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A48" s="12" t="s">
         <v>116</v>
       </c>
@@ -11372,7 +11372,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="49" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="49" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A49" s="12" t="s">
         <v>101</v>
       </c>
@@ -11545,7 +11545,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="50" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="50" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A50" s="11" t="s">
         <v>350</v>
       </c>
@@ -11718,7 +11718,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="51" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="51" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A51" s="11" t="s">
         <v>378</v>
       </c>
@@ -11891,7 +11891,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="52" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="52" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A52" s="11" t="s">
         <v>328</v>
       </c>
@@ -12064,7 +12064,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="53" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="53" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A53" s="12" t="s">
         <v>160</v>
       </c>
@@ -12237,7 +12237,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="54" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="54" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A54" s="12" t="s">
         <v>9</v>
       </c>
@@ -12410,7 +12410,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="55" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="55" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A55" s="12" t="s">
         <v>130</v>
       </c>
@@ -12583,7 +12583,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="56" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="56" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A56" s="12" t="s">
         <v>11</v>
       </c>
@@ -12756,7 +12756,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="57" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="57" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A57" s="12" t="s">
         <v>21</v>
       </c>
@@ -12929,7 +12929,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="58" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="58" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A58" s="12" t="s">
         <v>69</v>
       </c>
@@ -13102,7 +13102,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="59" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="59" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A59" s="12" t="s">
         <v>140</v>
       </c>
@@ -13275,7 +13275,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="60" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="60" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A60" s="11" t="s">
         <v>342</v>
       </c>
@@ -13448,7 +13448,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="61" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="61" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A61" s="11" t="s">
         <v>310</v>
       </c>
@@ -13621,7 +13621,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="62" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="62" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A62" s="12" t="s">
         <v>150</v>
       </c>
@@ -13794,7 +13794,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="63" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="63" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A63" s="12" t="s">
         <v>186</v>
       </c>
@@ -13967,7 +13967,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="64" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="64" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A64" s="12" t="s">
         <v>19</v>
       </c>
@@ -14140,7 +14140,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="65" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="65" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A65" s="11" t="s">
         <v>374</v>
       </c>
@@ -14313,7 +14313,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="66" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="66" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A66" s="12" t="s">
         <v>37</v>
       </c>
@@ -14486,7 +14486,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="67" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="67" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A67" s="12" t="s">
         <v>124</v>
       </c>
@@ -14659,7 +14659,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="68" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="68" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A68" s="11" t="s">
         <v>254</v>
       </c>
@@ -14832,7 +14832,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="69" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="69" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A69" s="12" t="s">
         <v>164</v>
       </c>
@@ -15005,7 +15005,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="70" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="70" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A70" s="12" t="s">
         <v>7</v>
       </c>
@@ -15178,7 +15178,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="71" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="71" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A71" s="11" t="s">
         <v>316</v>
       </c>
@@ -15351,7 +15351,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="72" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="72" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A72" s="12" t="s">
         <v>154</v>
       </c>
@@ -15524,7 +15524,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="73" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="73" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A73" s="12" t="s">
         <v>91</v>
       </c>
@@ -15697,7 +15697,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="74" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="74" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A74" s="12" t="s">
         <v>43</v>
       </c>
@@ -15870,7 +15870,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="75" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="75" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A75" s="12" t="s">
         <v>89</v>
       </c>
@@ -16043,7 +16043,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="76" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="76" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A76" s="12" t="s">
         <v>156</v>
       </c>
@@ -16216,7 +16216,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="77" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="77" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A77" s="12" t="s">
         <v>180</v>
       </c>
@@ -16389,7 +16389,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="78" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="78" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A78" s="13" t="s">
         <v>278</v>
       </c>
@@ -16562,7 +16562,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="79" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="79" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A79" s="11" t="s">
         <v>224</v>
       </c>
@@ -16735,7 +16735,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="80" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="80" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A80" s="13" t="s">
         <v>220</v>
       </c>
@@ -16908,7 +16908,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="81" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="81" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A81" s="11" t="s">
         <v>324</v>
       </c>
@@ -17081,7 +17081,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="82" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="82" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A82" s="13" t="s">
         <v>194</v>
       </c>
@@ -17254,7 +17254,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="83" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="83" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A83" s="12" t="s">
         <v>184</v>
       </c>
@@ -17427,7 +17427,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="84" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="84" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A84" s="13" t="s">
         <v>222</v>
       </c>
@@ -17600,7 +17600,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="85" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="85" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A85" s="11" t="s">
         <v>376</v>
       </c>
@@ -17773,7 +17773,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="86" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="86" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A86" s="12" t="s">
         <v>13</v>
       </c>
@@ -17946,7 +17946,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="87" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="87" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A87" s="12" t="s">
         <v>93</v>
       </c>
@@ -18119,7 +18119,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="88" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="88" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A88" s="12" t="s">
         <v>63</v>
       </c>
@@ -18292,7 +18292,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="89" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="89" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A89" s="11" t="s">
         <v>270</v>
       </c>
@@ -18465,7 +18465,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="90" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="90" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A90" s="13" t="s">
         <v>198</v>
       </c>
@@ -18638,7 +18638,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="91" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="91" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A91" s="11" t="s">
         <v>356</v>
       </c>
@@ -18811,7 +18811,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="92" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="92" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A92" s="11" t="s">
         <v>314</v>
       </c>
@@ -18984,7 +18984,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="93" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="93" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A93" s="11" t="s">
         <v>366</v>
       </c>
@@ -19157,7 +19157,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="94" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="94" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A94" s="12" t="s">
         <v>146</v>
       </c>
@@ -19330,7 +19330,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="95" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="95" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A95" s="11" t="s">
         <v>326</v>
       </c>
@@ -19503,7 +19503,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="96" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="96" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A96" s="12" t="s">
         <v>23</v>
       </c>
@@ -19676,7 +19676,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="97" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="97" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A97" s="12" t="s">
         <v>65</v>
       </c>
@@ -19849,7 +19849,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="98" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="98" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A98" s="11" t="s">
         <v>370</v>
       </c>
@@ -20022,7 +20022,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="99" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="99" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A99" s="13" t="s">
         <v>190</v>
       </c>
@@ -20195,7 +20195,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="100" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="100" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A100" s="13" t="s">
         <v>290</v>
       </c>
@@ -20368,7 +20368,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="101" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="101" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A101" s="12" t="s">
         <v>49</v>
       </c>
@@ -20541,7 +20541,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="102" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="102" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A102" s="12" t="s">
         <v>148</v>
       </c>
@@ -20714,7 +20714,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="103" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="103" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A103" s="13" t="s">
         <v>362</v>
       </c>
@@ -20887,7 +20887,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="104" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="104" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A104" s="13" t="s">
         <v>272</v>
       </c>
@@ -21060,7 +21060,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="105" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="105" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A105" s="12" t="s">
         <v>176</v>
       </c>
@@ -21233,7 +21233,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="106" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="106" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A106" s="11" t="s">
         <v>304</v>
       </c>
@@ -21406,7 +21406,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="107" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="107" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A107" s="12" t="s">
         <v>27</v>
       </c>
@@ -21579,7 +21579,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="108" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="108" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A108" s="11" t="s">
         <v>364</v>
       </c>
@@ -21752,7 +21752,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="109" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="109" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A109" s="12" t="s">
         <v>97</v>
       </c>
@@ -21925,7 +21925,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="110" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="110" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A110" s="12" t="s">
         <v>77</v>
       </c>
@@ -22098,7 +22098,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="111" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="111" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A111" s="11" t="s">
         <v>250</v>
       </c>
@@ -22271,7 +22271,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="112" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="112" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A112" s="11" t="s">
         <v>246</v>
       </c>
@@ -22444,7 +22444,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="113" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="113" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A113" s="12" t="s">
         <v>142</v>
       </c>
@@ -22617,7 +22617,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="114" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="114" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A114" s="12" t="s">
         <v>182</v>
       </c>
@@ -22790,7 +22790,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="115" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="115" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A115" s="13" t="s">
         <v>294</v>
       </c>
@@ -22963,7 +22963,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="116" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="116" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A116" s="12" t="s">
         <v>45</v>
       </c>
@@ -23136,7 +23136,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="117" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="117" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A117" s="13" t="s">
         <v>332</v>
       </c>
@@ -23309,7 +23309,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="118" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="118" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A118" s="13" t="s">
         <v>300</v>
       </c>
@@ -23482,7 +23482,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="119" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="119" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A119" s="12" t="s">
         <v>75</v>
       </c>
@@ -23655,7 +23655,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="120" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="120" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A120" s="12" t="s">
         <v>29</v>
       </c>
@@ -23828,7 +23828,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="121" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="121" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A121" s="12" t="s">
         <v>166</v>
       </c>
@@ -24001,7 +24001,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="122" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="122" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A122" s="12" t="s">
         <v>162</v>
       </c>
@@ -24174,7 +24174,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="123" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="123" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A123" s="12" t="s">
         <v>33</v>
       </c>
@@ -24347,7 +24347,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="124" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="124" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A124" s="13" t="s">
         <v>192</v>
       </c>
@@ -24520,7 +24520,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="125" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="125" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A125" s="13" t="s">
         <v>208</v>
       </c>
@@ -24693,7 +24693,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="126" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="126" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A126" s="12" t="s">
         <v>174</v>
       </c>
@@ -24866,7 +24866,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="127" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="127" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A127" s="12" t="s">
         <v>35</v>
       </c>
@@ -25039,7 +25039,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="128" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="128" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A128" s="11" t="s">
         <v>262</v>
       </c>
@@ -25212,7 +25212,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="129" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="129" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A129" s="12" t="s">
         <v>67</v>
       </c>
@@ -25385,7 +25385,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="130" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="130" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A130" s="11" t="s">
         <v>242</v>
       </c>
@@ -25558,7 +25558,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="131" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="131" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A131" s="13" t="s">
         <v>296</v>
       </c>
@@ -25731,7 +25731,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="132" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="132" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A132" s="12" t="s">
         <v>53</v>
       </c>
@@ -25904,7 +25904,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="133" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="133" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A133" s="11" t="s">
         <v>352</v>
       </c>
@@ -26077,7 +26077,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="134" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="134" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A134" s="12" t="s">
         <v>25</v>
       </c>
@@ -26250,7 +26250,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="135" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="135" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A135" s="11" t="s">
         <v>340</v>
       </c>
@@ -26423,7 +26423,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="136" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="136" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A136" s="12" t="s">
         <v>83</v>
       </c>
@@ -26596,7 +26596,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="137" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="137" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A137" s="13" t="s">
         <v>338</v>
       </c>
@@ -26769,7 +26769,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="138" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="138" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A138" s="12" t="s">
         <v>59</v>
       </c>
@@ -26942,7 +26942,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="139" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="139" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A139" s="11" t="s">
         <v>248</v>
       </c>
@@ -27115,7 +27115,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="140" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="140" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A140" s="12" t="s">
         <v>132</v>
       </c>
@@ -27288,7 +27288,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="141" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="141" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A141" s="11" t="s">
         <v>360</v>
       </c>
@@ -27461,7 +27461,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="142" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="142" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A142" s="11" t="s">
         <v>306</v>
       </c>
@@ -27634,7 +27634,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="143" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="143" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A143" s="11" t="s">
         <v>232</v>
       </c>
@@ -27807,7 +27807,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="144" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="144" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A144" s="13" t="s">
         <v>214</v>
       </c>
@@ -27980,7 +27980,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="145" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="145" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A145" s="12" t="s">
         <v>47</v>
       </c>
@@ -28153,7 +28153,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="146" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="146" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A146" s="12" t="s">
         <v>51</v>
       </c>
@@ -28326,7 +28326,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="147" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="147" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A147" s="12" t="s">
         <v>41</v>
       </c>
@@ -28499,7 +28499,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="148" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="148" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A148" s="12" t="s">
         <v>99</v>
       </c>
@@ -28672,7 +28672,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="149" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="149" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A149" s="12" t="s">
         <v>81</v>
       </c>
@@ -28845,7 +28845,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="150" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="150" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A150" s="11" t="s">
         <v>322</v>
       </c>
@@ -29018,7 +29018,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="151" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="151" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A151" s="11" t="s">
         <v>238</v>
       </c>
@@ -29191,7 +29191,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="152" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="152" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A152" s="12" t="s">
         <v>138</v>
       </c>
@@ -29364,7 +29364,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="153" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="153" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A153" s="11" t="s">
         <v>256</v>
       </c>
@@ -29537,7 +29537,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="154" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="154" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A154" s="12" t="s">
         <v>71</v>
       </c>
@@ -29710,7 +29710,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="155" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="155" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A155" s="11" t="s">
         <v>258</v>
       </c>
@@ -29883,7 +29883,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="156" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="156" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A156" s="13" t="s">
         <v>302</v>
       </c>
@@ -30056,7 +30056,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="157" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="157" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A157" s="12" t="s">
         <v>107</v>
       </c>
@@ -30229,7 +30229,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="158" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="158" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A158" s="11" t="s">
         <v>268</v>
       </c>
@@ -30402,7 +30402,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="159" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="159" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A159" s="12" t="s">
         <v>31</v>
       </c>
@@ -30575,7 +30575,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="160" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="160" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A160" s="12" t="s">
         <v>110</v>
       </c>
@@ -30748,7 +30748,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="161" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="161" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A161" s="11" t="s">
         <v>234</v>
       </c>
@@ -30921,7 +30921,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="162" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="162" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A162" s="13" t="s">
         <v>276</v>
       </c>
@@ -31094,7 +31094,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="163" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="163" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A163" s="11" t="s">
         <v>354</v>
       </c>
@@ -31267,7 +31267,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="164" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="164" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A164" s="12" t="s">
         <v>95</v>
       </c>
@@ -31440,7 +31440,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="165" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="165" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A165" s="12" t="s">
         <v>15</v>
       </c>
@@ -31613,7 +31613,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="166" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="166" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A166" s="13" t="s">
         <v>196</v>
       </c>
@@ -31786,7 +31786,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="167" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="167" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A167" s="12" t="s">
         <v>79</v>
       </c>
@@ -31959,7 +31959,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="168" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="168" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A168" s="12" t="s">
         <v>112</v>
       </c>
@@ -32132,7 +32132,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="169" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="169" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A169" s="12" t="s">
         <v>136</v>
       </c>
@@ -32305,7 +32305,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="170" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="170" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A170" s="13" t="s">
         <v>204</v>
       </c>
@@ -32478,7 +32478,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="171" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="171" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A171" s="12" t="s">
         <v>134</v>
       </c>
@@ -32651,7 +32651,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="172" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="172" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A172" s="13" t="s">
         <v>202</v>
       </c>
@@ -32824,7 +32824,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="173" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="173" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A173" s="12" t="s">
         <v>170</v>
       </c>
@@ -32997,7 +32997,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="174" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="174" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A174" s="11" t="s">
         <v>228</v>
       </c>
@@ -33170,7 +33170,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="175" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="175" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A175" s="13" t="s">
         <v>344</v>
       </c>
@@ -33343,7 +33343,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="176" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="176" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A176" s="13" t="s">
         <v>200</v>
       </c>
@@ -33516,7 +33516,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="177" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="177" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A177" s="11" t="s">
         <v>236</v>
       </c>
@@ -33689,7 +33689,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="178" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="178" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A178" s="11" t="s">
         <v>260</v>
       </c>
@@ -33862,7 +33862,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="179" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="179" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A179" s="12" t="s">
         <v>57</v>
       </c>
@@ -34035,7 +34035,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="180" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="180" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A180" s="12" t="s">
         <v>114</v>
       </c>
@@ -34208,7 +34208,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="181" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="181" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A181" s="12" t="s">
         <v>122</v>
       </c>
@@ -34381,7 +34381,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="182" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="182" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A182" s="13" t="s">
         <v>334</v>
       </c>
@@ -34554,7 +34554,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="183" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="183" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A183" s="12" t="s">
         <v>105</v>
       </c>
@@ -34727,7 +34727,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="184" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="184" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A184" s="12" t="s">
         <v>152</v>
       </c>
@@ -34900,7 +34900,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="185" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="185" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A185" s="12" t="s">
         <v>61</v>
       </c>
@@ -35073,7 +35073,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="186" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="186" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A186" s="12" t="s">
         <v>73</v>
       </c>
@@ -35246,7 +35246,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="187" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="187" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A187" s="12" t="s">
         <v>85</v>
       </c>
@@ -35419,7 +35419,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="188" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="188" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A188" s="13" t="s">
         <v>298</v>
       </c>
@@ -35592,7 +35592,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="189" spans="1:57" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="189" spans="1:57" ht="20.100000000000001" customHeight="1">
       <c r="A189" s="13" t="s">
         <v>282</v>
       </c>
@@ -35770,7 +35770,7 @@
     <sortCondition ref="AP2:AP189"/>
   </sortState>
   <phoneticPr fontId="2" type="noConversion"/>
-  <conditionalFormatting sqref="AW1:AW1048576 AY1:AY1048576 BC1:BC1048576 BA1:BA1048576">
+  <conditionalFormatting sqref="AW1:AW1048576 AY1:AY1048576 BA1:BA1048576 BC1:BC1048576">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
       <formula>0.05</formula>
     </cfRule>
@@ -35791,17 +35791,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35B128DD-DA5B-5943-9431-35A61A644B69}">
   <dimension ref="A1:BD16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="20.100000000000001" customHeight="1"/>
   <cols>
     <col min="2" max="3" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="69.33203125" customWidth="1"/>
-    <col min="6" max="23" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="69.28515625" customWidth="1"/>
+    <col min="6" max="23" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="24" max="41" width="11" bestFit="1" customWidth="1"/>
     <col min="43" max="56" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
@@ -35971,7 +35971,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="2" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A2" s="37" t="s">
         <v>43</v>
       </c>
@@ -36141,7 +36141,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="3" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A3" s="37" t="s">
         <v>244</v>
       </c>
@@ -36311,7 +36311,7 @@
         <v>0.19</v>
       </c>
     </row>
-    <row r="4" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A4" s="39" t="s">
         <v>318</v>
       </c>
@@ -36481,7 +36481,7 @@
         <v>0.11</v>
       </c>
     </row>
-    <row r="5" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A5" s="39" t="s">
         <v>206</v>
       </c>
@@ -36651,7 +36651,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="6" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A6" s="39" t="s">
         <v>37</v>
       </c>
@@ -36821,7 +36821,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="7" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A7" s="37" t="s">
         <v>208</v>
       </c>
@@ -36991,7 +36991,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="8" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A8" s="37" t="s">
         <v>134</v>
       </c>
@@ -37161,7 +37161,7 @@
         <v>0.11</v>
       </c>
     </row>
-    <row r="9" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A9" s="37" t="s">
         <v>45</v>
       </c>
@@ -37331,7 +37331,7 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="10" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A10" s="37" t="s">
         <v>232</v>
       </c>
@@ -37501,7 +37501,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="11" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A11" s="37" t="s">
         <v>330</v>
       </c>
@@ -37671,7 +37671,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="12" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A12" s="39" t="s">
         <v>246</v>
       </c>
@@ -37841,7 +37841,7 @@
         <v>0.08</v>
       </c>
     </row>
-    <row r="13" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A13" s="37" t="s">
         <v>105</v>
       </c>
@@ -38011,7 +38011,7 @@
         <v>0.27</v>
       </c>
     </row>
-    <row r="14" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A14" s="37" t="s">
         <v>118</v>
       </c>
@@ -38181,7 +38181,7 @@
         <v>0.17</v>
       </c>
     </row>
-    <row r="15" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A15" s="37" t="s">
         <v>79</v>
       </c>
@@ -38351,7 +38351,7 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A16" s="37" t="s">
         <v>372</v>
       </c>
@@ -38529,21 +38529,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE3378BC-7E7F-A547-A7C0-185E9AAFDD83}">
   <dimension ref="A1:BD42"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="20.100000000000001" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" style="37"/>
-    <col min="2" max="3" width="11.1640625" style="37" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.6640625" style="37" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="100.6640625" style="37" customWidth="1"/>
-    <col min="6" max="23" width="11.6640625" style="37" bestFit="1" customWidth="1"/>
-    <col min="24" max="41" width="11.83203125" style="37" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="10.83203125" style="37"/>
-    <col min="43" max="48" width="11.83203125" style="37" bestFit="1" customWidth="1"/>
-    <col min="49" max="56" width="11.1640625" style="37" bestFit="1" customWidth="1"/>
-    <col min="57" max="16384" width="10.83203125" style="37"/>
+    <col min="1" max="1" width="10.85546875" style="37"/>
+    <col min="2" max="3" width="11.140625" style="37" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" style="37" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="100.7109375" style="37" customWidth="1"/>
+    <col min="6" max="23" width="11.7109375" style="37" bestFit="1" customWidth="1"/>
+    <col min="24" max="41" width="11.85546875" style="37" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="10.85546875" style="37"/>
+    <col min="43" max="48" width="11.85546875" style="37" bestFit="1" customWidth="1"/>
+    <col min="49" max="56" width="11.140625" style="37" bestFit="1" customWidth="1"/>
+    <col min="57" max="16384" width="10.85546875" style="37"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
@@ -38713,7 +38713,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="2" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A2" s="39" t="s">
         <v>33</v>
       </c>
@@ -38883,7 +38883,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="3" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A3" s="39" t="s">
         <v>37</v>
       </c>
@@ -39053,7 +39053,7 @@
         <v>7.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A4" s="39" t="s">
         <v>59</v>
       </c>
@@ -39223,7 +39223,7 @@
         <v>5.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A5" s="39" t="s">
         <v>368</v>
       </c>
@@ -39393,7 +39393,7 @@
         <v>8.6999999999999994E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A6" s="39" t="s">
         <v>110</v>
       </c>
@@ -39563,7 +39563,7 @@
         <v>6.7000000000000004E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A7" s="39" t="s">
         <v>228</v>
       </c>
@@ -39733,7 +39733,7 @@
         <v>7.3999999999999996E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A8" s="39" t="s">
         <v>330</v>
       </c>
@@ -39903,7 +39903,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A9" s="39" t="s">
         <v>208</v>
       </c>
@@ -40073,7 +40073,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A10" s="39" t="s">
         <v>354</v>
       </c>
@@ -40243,7 +40243,7 @@
         <v>3.2000000000000001E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A11" s="39" t="s">
         <v>103</v>
       </c>
@@ -40413,7 +40413,7 @@
         <v>5.0999999999999997E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A12" s="39" t="s">
         <v>230</v>
       </c>
@@ -40583,7 +40583,7 @@
         <v>5.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A13" s="39" t="s">
         <v>280</v>
       </c>
@@ -40753,7 +40753,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A14" s="39" t="s">
         <v>172</v>
       </c>
@@ -40923,7 +40923,7 @@
         <v>0.42899999999999999</v>
       </c>
     </row>
-    <row r="15" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A15" s="39" t="s">
         <v>55</v>
       </c>
@@ -41093,7 +41093,7 @@
         <v>2.3E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A16" s="39" t="s">
         <v>222</v>
       </c>
@@ -41263,7 +41263,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A17" s="39" t="s">
         <v>7</v>
       </c>
@@ -41433,7 +41433,7 @@
         <v>0.317</v>
       </c>
     </row>
-    <row r="18" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A18" s="39" t="s">
         <v>318</v>
       </c>
@@ -41603,7 +41603,7 @@
         <v>3.2000000000000001E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A19" s="39" t="s">
         <v>246</v>
       </c>
@@ -41773,7 +41773,7 @@
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A20" s="39" t="s">
         <v>366</v>
       </c>
@@ -41943,7 +41943,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A21" s="39" t="s">
         <v>41</v>
       </c>
@@ -42113,7 +42113,7 @@
         <v>5.0999999999999997E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A22" s="39" t="s">
         <v>156</v>
       </c>
@@ -42283,7 +42283,7 @@
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="23" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A23" s="39" t="s">
         <v>65</v>
       </c>
@@ -42453,7 +42453,7 @@
         <v>7.6999999999999999E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A24" s="39" t="s">
         <v>184</v>
       </c>
@@ -42623,7 +42623,7 @@
         <v>0.46600000000000003</v>
       </c>
     </row>
-    <row r="25" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A25" s="39" t="s">
         <v>206</v>
       </c>
@@ -42793,7 +42793,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A26" s="39" t="s">
         <v>428</v>
       </c>
@@ -42963,7 +42963,7 @@
         <v>0.126</v>
       </c>
     </row>
-    <row r="27" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A27" s="39" t="s">
         <v>99</v>
       </c>
@@ -43133,7 +43133,7 @@
         <v>3.3000000000000002E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A28" s="39" t="s">
         <v>232</v>
       </c>
@@ -43303,7 +43303,7 @@
         <v>0.23599999999999999</v>
       </c>
     </row>
-    <row r="29" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A29" s="39" t="s">
         <v>49</v>
       </c>
@@ -43473,7 +43473,7 @@
         <v>0.14699999999999999</v>
       </c>
     </row>
-    <row r="30" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A30" s="39" t="s">
         <v>105</v>
       </c>
@@ -43643,7 +43643,7 @@
         <v>4.7E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A31" s="39" t="s">
         <v>220</v>
       </c>
@@ -43813,7 +43813,7 @@
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="32" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A32" s="39" t="s">
         <v>45</v>
       </c>
@@ -43983,7 +43983,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="33" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A33" s="39" t="s">
         <v>234</v>
       </c>
@@ -44153,7 +44153,7 @@
         <v>4.2999999999999997E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A34" s="39" t="s">
         <v>274</v>
       </c>
@@ -44323,7 +44323,7 @@
         <v>0.11600000000000001</v>
       </c>
     </row>
-    <row r="35" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A35" s="39" t="s">
         <v>134</v>
       </c>
@@ -44493,7 +44493,7 @@
         <v>0.32</v>
       </c>
     </row>
-    <row r="36" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A36" s="39" t="s">
         <v>288</v>
       </c>
@@ -44663,7 +44663,7 @@
         <v>0.11799999999999999</v>
       </c>
     </row>
-    <row r="37" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A37" s="39" t="s">
         <v>130</v>
       </c>
@@ -44833,7 +44833,7 @@
         <v>0.27500000000000002</v>
       </c>
     </row>
-    <row r="38" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A38" s="39" t="s">
         <v>264</v>
       </c>
@@ -45003,7 +45003,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="39" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A39" s="39" t="s">
         <v>27</v>
       </c>
@@ -45173,7 +45173,7 @@
         <v>0.42399999999999999</v>
       </c>
     </row>
-    <row r="40" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A40" s="39" t="s">
         <v>244</v>
       </c>
@@ -45343,7 +45343,7 @@
         <v>0.38400000000000001</v>
       </c>
     </row>
-    <row r="41" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="41" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A41" s="39" t="s">
         <v>43</v>
       </c>
@@ -45513,7 +45513,7 @@
         <v>0.373</v>
       </c>
     </row>
-    <row r="42" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="42" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A42" s="39" t="s">
         <v>270</v>
       </c>
@@ -45691,12 +45691,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84E5A52D-7F82-124D-A2A5-7137552E0378}">
   <dimension ref="A1:BN135"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="20.100000000000001" customHeight="1"/>
   <cols>
-    <col min="1" max="16384" width="10.83203125" style="37"/>
+    <col min="1" max="16384" width="10.85546875" style="37"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A1" s="37" t="s">
         <v>0</v>
       </c>
@@ -45896,7 +45896,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="2" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A2" s="37" t="s">
         <v>126</v>
       </c>
@@ -46096,7 +46096,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="3" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A3" s="37" t="s">
         <v>284</v>
       </c>
@@ -46296,7 +46296,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="4" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A4" s="37" t="s">
         <v>348</v>
       </c>
@@ -46496,7 +46496,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="5" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A5" s="37" t="s">
         <v>144</v>
       </c>
@@ -46696,7 +46696,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="6" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A6" s="37" t="s">
         <v>346</v>
       </c>
@@ -46896,7 +46896,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="7" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A7" s="37" t="s">
         <v>39</v>
       </c>
@@ -47096,7 +47096,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A8" s="37" t="s">
         <v>266</v>
       </c>
@@ -47296,7 +47296,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="9" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A9" s="37" t="s">
         <v>87</v>
       </c>
@@ -47496,7 +47496,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="10" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A10" s="37" t="s">
         <v>103</v>
       </c>
@@ -47696,7 +47696,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="11" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A11" s="37" t="s">
         <v>109</v>
       </c>
@@ -47896,7 +47896,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="12" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A12" s="37" t="s">
         <v>218</v>
       </c>
@@ -48096,7 +48096,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="13" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A13" s="37" t="s">
         <v>178</v>
       </c>
@@ -48296,7 +48296,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="14" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A14" s="37" t="s">
         <v>158</v>
       </c>
@@ -48496,7 +48496,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="15" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A15" s="37" t="s">
         <v>230</v>
       </c>
@@ -48696,7 +48696,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="16" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A16" s="37" t="s">
         <v>206</v>
       </c>
@@ -48896,7 +48896,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="17" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A17" s="37" t="s">
         <v>318</v>
       </c>
@@ -49096,7 +49096,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="18" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A18" s="37" t="s">
         <v>336</v>
       </c>
@@ -49296,7 +49296,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="19" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A19" s="37" t="s">
         <v>264</v>
       </c>
@@ -49496,7 +49496,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="20" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A20" s="37" t="s">
         <v>432</v>
       </c>
@@ -49696,7 +49696,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="21" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A21" s="37" t="s">
         <v>128</v>
       </c>
@@ -49896,7 +49896,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="22" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A22" s="37" t="s">
         <v>118</v>
       </c>
@@ -50096,7 +50096,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="23" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A23" s="37" t="s">
         <v>312</v>
       </c>
@@ -50296,7 +50296,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="24" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A24" s="37" t="s">
         <v>244</v>
       </c>
@@ -50496,7 +50496,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="25" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A25" s="37" t="s">
         <v>55</v>
       </c>
@@ -50696,7 +50696,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="26" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A26" s="37" t="s">
         <v>368</v>
       </c>
@@ -50896,7 +50896,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="27" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A27" s="37" t="s">
         <v>434</v>
       </c>
@@ -51096,7 +51096,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="28" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A28" s="37" t="s">
         <v>358</v>
       </c>
@@ -51296,7 +51296,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="29" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A29" s="37" t="s">
         <v>168</v>
       </c>
@@ -51496,7 +51496,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="30" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A30" s="37" t="s">
         <v>280</v>
       </c>
@@ -51696,7 +51696,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="31" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A31" s="37" t="s">
         <v>116</v>
       </c>
@@ -51896,7 +51896,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="32" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A32" s="37" t="s">
         <v>101</v>
       </c>
@@ -52096,7 +52096,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="33" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A33" s="37" t="s">
         <v>350</v>
       </c>
@@ -52296,7 +52296,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="34" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A34" s="37" t="s">
         <v>328</v>
       </c>
@@ -52496,7 +52496,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="35" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A35" s="37" t="s">
         <v>9</v>
       </c>
@@ -52696,7 +52696,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="36" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A36" s="37" t="s">
         <v>130</v>
       </c>
@@ -52896,7 +52896,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="37" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A37" s="37" t="s">
         <v>140</v>
       </c>
@@ -53096,7 +53096,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="38" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A38" s="37" t="s">
         <v>342</v>
       </c>
@@ -53296,7 +53296,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="39" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A39" s="37" t="s">
         <v>436</v>
       </c>
@@ -53496,7 +53496,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="40" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A40" s="37" t="s">
         <v>310</v>
       </c>
@@ -53696,7 +53696,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="41" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="41" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A41" s="37" t="s">
         <v>186</v>
       </c>
@@ -53896,7 +53896,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="42" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="42" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A42" s="37" t="s">
         <v>37</v>
       </c>
@@ -54096,7 +54096,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="43" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A43" s="37" t="s">
         <v>124</v>
       </c>
@@ -54296,7 +54296,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="44" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="44" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A44" s="37" t="s">
         <v>438</v>
       </c>
@@ -54496,7 +54496,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="45" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="45" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A45" s="37" t="s">
         <v>164</v>
       </c>
@@ -54696,7 +54696,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="46" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="46" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A46" s="37" t="s">
         <v>316</v>
       </c>
@@ -54896,7 +54896,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="47" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="47" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A47" s="37" t="s">
         <v>91</v>
       </c>
@@ -55096,7 +55096,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="48" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="48" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A48" s="37" t="s">
         <v>43</v>
       </c>
@@ -55296,7 +55296,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="49" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="49" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A49" s="37" t="s">
         <v>156</v>
       </c>
@@ -55496,7 +55496,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="50" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="50" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A50" s="37" t="s">
         <v>180</v>
       </c>
@@ -55696,7 +55696,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="51" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="51" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A51" s="37" t="s">
         <v>440</v>
       </c>
@@ -55896,7 +55896,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="52" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="52" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A52" s="37" t="s">
         <v>278</v>
       </c>
@@ -56096,7 +56096,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="53" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="53" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A53" s="37" t="s">
         <v>220</v>
       </c>
@@ -56296,7 +56296,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="54" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="54" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A54" s="37" t="s">
         <v>442</v>
       </c>
@@ -56496,7 +56496,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="55" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="55" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A55" s="37" t="s">
         <v>194</v>
       </c>
@@ -56696,7 +56696,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="56" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="56" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A56" s="37" t="s">
         <v>184</v>
       </c>
@@ -56896,7 +56896,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="57" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="57" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A57" s="37" t="s">
         <v>222</v>
       </c>
@@ -57096,7 +57096,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="58" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="58" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A58" s="37" t="s">
         <v>376</v>
       </c>
@@ -57296,7 +57296,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="59" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="59" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A59" s="37" t="s">
         <v>444</v>
       </c>
@@ -57496,7 +57496,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="60" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="60" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A60" s="37" t="s">
         <v>446</v>
       </c>
@@ -57696,7 +57696,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="61" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="61" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A61" s="37" t="s">
         <v>93</v>
       </c>
@@ -57896,7 +57896,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="62" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="62" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A62" s="37" t="s">
         <v>63</v>
       </c>
@@ -58096,7 +58096,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="63" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="63" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A63" s="37" t="s">
         <v>448</v>
       </c>
@@ -58296,7 +58296,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="64" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="64" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A64" s="37" t="s">
         <v>198</v>
       </c>
@@ -58496,7 +58496,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="65" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="65" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A65" s="37" t="s">
         <v>314</v>
       </c>
@@ -58696,7 +58696,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="66" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="66" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A66" s="37" t="s">
         <v>366</v>
       </c>
@@ -58896,7 +58896,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="67" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="67" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A67" s="37" t="s">
         <v>146</v>
       </c>
@@ -59096,7 +59096,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="68" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="68" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A68" s="37" t="s">
         <v>23</v>
       </c>
@@ -59296,7 +59296,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="69" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="69" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A69" s="37" t="s">
         <v>190</v>
       </c>
@@ -59496,7 +59496,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="70" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="70" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A70" s="37" t="s">
         <v>290</v>
       </c>
@@ -59696,7 +59696,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="71" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="71" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A71" s="37" t="s">
         <v>450</v>
       </c>
@@ -59896,7 +59896,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="72" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="72" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A72" s="37" t="s">
         <v>49</v>
       </c>
@@ -60096,7 +60096,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="73" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="73" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A73" s="37" t="s">
         <v>148</v>
       </c>
@@ -60296,7 +60296,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="74" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="74" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A74" s="37" t="s">
         <v>362</v>
       </c>
@@ -60496,7 +60496,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="75" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="75" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A75" s="37" t="s">
         <v>452</v>
       </c>
@@ -60696,7 +60696,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="76" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="76" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A76" s="37" t="s">
         <v>27</v>
       </c>
@@ -60896,7 +60896,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="77" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="77" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A77" s="37" t="s">
         <v>364</v>
       </c>
@@ -61096,7 +61096,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="78" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="78" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A78" s="37" t="s">
         <v>77</v>
       </c>
@@ -61296,7 +61296,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="79" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="79" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A79" s="37" t="s">
         <v>246</v>
       </c>
@@ -61496,7 +61496,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="80" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="80" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A80" s="37" t="s">
         <v>182</v>
       </c>
@@ -61696,7 +61696,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="81" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="81" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A81" s="37" t="s">
         <v>294</v>
       </c>
@@ -61896,7 +61896,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="82" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="82" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A82" s="37" t="s">
         <v>45</v>
       </c>
@@ -62096,7 +62096,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="83" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="83" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A83" s="37" t="s">
         <v>75</v>
       </c>
@@ -62296,7 +62296,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="84" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="84" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A84" s="37" t="s">
         <v>29</v>
       </c>
@@ -62496,7 +62496,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="85" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="85" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A85" s="37" t="s">
         <v>166</v>
       </c>
@@ -62696,7 +62696,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="86" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="86" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A86" s="37" t="s">
         <v>162</v>
       </c>
@@ -62896,7 +62896,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="87" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="87" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A87" s="37" t="s">
         <v>33</v>
       </c>
@@ -63096,7 +63096,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="88" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="88" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A88" s="37" t="s">
         <v>454</v>
       </c>
@@ -63296,7 +63296,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="89" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="89" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A89" s="37" t="s">
         <v>208</v>
       </c>
@@ -63496,7 +63496,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="90" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="90" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A90" s="37" t="s">
         <v>456</v>
       </c>
@@ -63696,7 +63696,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="91" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="91" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A91" s="37" t="s">
         <v>262</v>
       </c>
@@ -63896,7 +63896,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="92" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="92" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A92" s="37" t="s">
         <v>242</v>
       </c>
@@ -64096,7 +64096,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="93" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="93" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A93" s="37" t="s">
         <v>53</v>
       </c>
@@ -64296,7 +64296,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="94" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="94" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A94" s="37" t="s">
         <v>352</v>
       </c>
@@ -64496,7 +64496,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="95" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="95" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A95" s="37" t="s">
         <v>25</v>
       </c>
@@ -64696,7 +64696,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="96" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="96" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A96" s="37" t="s">
         <v>340</v>
       </c>
@@ -64896,7 +64896,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="97" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="97" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A97" s="37" t="s">
         <v>83</v>
       </c>
@@ -65096,7 +65096,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="98" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="98" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A98" s="37" t="s">
         <v>338</v>
       </c>
@@ -65296,7 +65296,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="99" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="99" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A99" s="37" t="s">
         <v>59</v>
       </c>
@@ -65496,7 +65496,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="100" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="100" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A100" s="37" t="s">
         <v>306</v>
       </c>
@@ -65696,7 +65696,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="101" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="101" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A101" s="37" t="s">
         <v>232</v>
       </c>
@@ -65896,7 +65896,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="102" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="102" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A102" s="37" t="s">
         <v>214</v>
       </c>
@@ -66096,7 +66096,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="103" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="103" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A103" s="37" t="s">
         <v>47</v>
       </c>
@@ -66296,7 +66296,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="104" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="104" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A104" s="37" t="s">
         <v>51</v>
       </c>
@@ -66496,7 +66496,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="105" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="105" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A105" s="37" t="s">
         <v>458</v>
       </c>
@@ -66696,7 +66696,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="106" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="106" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A106" s="37" t="s">
         <v>41</v>
       </c>
@@ -66896,7 +66896,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="107" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="107" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A107" s="37" t="s">
         <v>460</v>
       </c>
@@ -67096,7 +67096,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="108" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="108" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A108" s="37" t="s">
         <v>99</v>
       </c>
@@ -67296,7 +67296,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="109" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="109" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A109" s="37" t="s">
         <v>238</v>
       </c>
@@ -67496,7 +67496,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="110" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="110" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A110" s="37" t="s">
         <v>138</v>
       </c>
@@ -67696,7 +67696,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="111" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="111" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A111" s="37" t="s">
         <v>71</v>
       </c>
@@ -67896,7 +67896,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="112" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="112" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A112" s="37" t="s">
         <v>302</v>
       </c>
@@ -68096,7 +68096,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="113" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="113" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A113" s="37" t="s">
         <v>462</v>
       </c>
@@ -68296,7 +68296,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="114" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="114" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A114" s="37" t="s">
         <v>268</v>
       </c>
@@ -68496,7 +68496,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="115" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="115" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A115" s="37" t="s">
         <v>31</v>
       </c>
@@ -68696,7 +68696,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="116" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="116" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A116" s="37" t="s">
         <v>234</v>
       </c>
@@ -68896,7 +68896,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="117" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="117" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A117" s="37" t="s">
         <v>354</v>
       </c>
@@ -69096,7 +69096,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="118" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="118" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A118" s="37" t="s">
         <v>95</v>
       </c>
@@ -69296,7 +69296,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="119" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="119" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A119" s="37" t="s">
         <v>15</v>
       </c>
@@ -69496,7 +69496,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="120" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="120" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A120" s="37" t="s">
         <v>134</v>
       </c>
@@ -69696,7 +69696,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="121" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="121" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A121" s="37" t="s">
         <v>202</v>
       </c>
@@ -69896,7 +69896,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="122" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="122" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A122" s="37" t="s">
         <v>228</v>
       </c>
@@ -70096,7 +70096,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="123" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="123" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A123" s="37" t="s">
         <v>344</v>
       </c>
@@ -70296,7 +70296,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="124" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="124" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A124" s="37" t="s">
         <v>200</v>
       </c>
@@ -70496,7 +70496,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="125" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="125" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A125" s="37" t="s">
         <v>236</v>
       </c>
@@ -70696,7 +70696,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="126" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="126" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A126" s="37" t="s">
         <v>114</v>
       </c>
@@ -70896,7 +70896,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="127" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="127" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A127" s="37" t="s">
         <v>122</v>
       </c>
@@ -71096,7 +71096,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="128" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="128" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A128" s="37" t="s">
         <v>334</v>
       </c>
@@ -71296,7 +71296,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="129" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="129" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A129" s="37" t="s">
         <v>105</v>
       </c>
@@ -71496,7 +71496,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="130" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="130" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A130" s="37" t="s">
         <v>152</v>
       </c>
@@ -71696,7 +71696,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="131" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="131" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A131" s="37" t="s">
         <v>61</v>
       </c>
@@ -71896,7 +71896,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="132" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="132" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A132" s="37" t="s">
         <v>464</v>
       </c>
@@ -72096,7 +72096,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="133" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="133" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A133" s="37" t="s">
         <v>85</v>
       </c>
@@ -72296,7 +72296,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="134" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="134" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A134" s="37" t="s">
         <v>298</v>
       </c>
@@ -72496,7 +72496,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="135" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="135" spans="1:66" ht="20.100000000000001" customHeight="1">
       <c r="A135" s="37" t="s">
         <v>466</v>
       </c>
@@ -72704,20 +72704,20 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB9BF4A6-C295-0442-9EAA-87EDB0F09D1D}">
   <dimension ref="A1:BD48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="20.100000000000001" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" style="37"/>
+    <col min="1" max="1" width="10.85546875" style="37"/>
     <col min="2" max="3" width="11" style="37" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.6640625" style="37" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="71.83203125" style="37" customWidth="1"/>
-    <col min="6" max="23" width="11.6640625" style="37" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" style="37" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="71.85546875" style="37" customWidth="1"/>
+    <col min="6" max="23" width="11.7109375" style="37" bestFit="1" customWidth="1"/>
     <col min="24" max="41" width="11" style="37" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="10.83203125" style="37"/>
+    <col min="42" max="42" width="10.85546875" style="37"/>
     <col min="43" max="56" width="11" style="37" bestFit="1" customWidth="1"/>
-    <col min="57" max="16384" width="10.83203125" style="37"/>
+    <col min="57" max="16384" width="10.85546875" style="37"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
@@ -72887,7 +72887,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="2" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A2" s="39" t="s">
         <v>306</v>
       </c>
@@ -73057,7 +73057,7 @@
         <v>0.22700000000000001</v>
       </c>
     </row>
-    <row r="3" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A3" s="39" t="s">
         <v>264</v>
       </c>
@@ -73227,7 +73227,7 @@
         <v>0.182</v>
       </c>
     </row>
-    <row r="4" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A4" s="39" t="s">
         <v>190</v>
       </c>
@@ -73397,7 +73397,7 @@
         <v>0.152</v>
       </c>
     </row>
-    <row r="5" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A5" s="39" t="s">
         <v>202</v>
       </c>
@@ -73567,7 +73567,7 @@
         <v>0.19500000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A6" s="39" t="s">
         <v>246</v>
       </c>
@@ -73737,7 +73737,7 @@
         <v>0.129</v>
       </c>
     </row>
-    <row r="7" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A7" s="39" t="s">
         <v>244</v>
       </c>
@@ -73907,7 +73907,7 @@
         <v>0.11</v>
       </c>
     </row>
-    <row r="8" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A8" s="39" t="s">
         <v>208</v>
       </c>
@@ -74077,7 +74077,7 @@
         <v>0.109</v>
       </c>
     </row>
-    <row r="9" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A9" s="39" t="s">
         <v>65</v>
       </c>
@@ -74247,7 +74247,7 @@
         <v>8.4000000000000005E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A10" s="39" t="s">
         <v>61</v>
       </c>
@@ -74417,7 +74417,7 @@
         <v>0.19400000000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A11" s="39" t="s">
         <v>99</v>
       </c>
@@ -74587,7 +74587,7 @@
         <v>0.16200000000000001</v>
       </c>
     </row>
-    <row r="12" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A12" s="39" t="s">
         <v>29</v>
       </c>
@@ -74757,7 +74757,7 @@
         <v>0.36499999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A13" s="39" t="s">
         <v>366</v>
       </c>
@@ -74927,7 +74927,7 @@
         <v>0.104</v>
       </c>
     </row>
-    <row r="14" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A14" s="39" t="s">
         <v>220</v>
       </c>
@@ -75097,7 +75097,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="15" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A15" s="39" t="s">
         <v>368</v>
       </c>
@@ -75267,7 +75267,7 @@
         <v>0.127</v>
       </c>
     </row>
-    <row r="16" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A16" s="39" t="s">
         <v>164</v>
       </c>
@@ -75437,7 +75437,7 @@
         <v>0.19700000000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A17" s="39" t="s">
         <v>59</v>
       </c>
@@ -75607,7 +75607,7 @@
         <v>0.246</v>
       </c>
     </row>
-    <row r="18" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A18" s="39" t="s">
         <v>73</v>
       </c>
@@ -75777,7 +75777,7 @@
         <v>1.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A19" s="39" t="s">
         <v>55</v>
       </c>
@@ -75947,7 +75947,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="20" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A20" s="39" t="s">
         <v>45</v>
       </c>
@@ -76117,7 +76117,7 @@
         <v>8.5999999999999993E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A21" s="39" t="s">
         <v>37</v>
       </c>
@@ -76287,7 +76287,7 @@
         <v>0.23599999999999999</v>
       </c>
     </row>
-    <row r="22" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A22" s="39" t="s">
         <v>304</v>
       </c>
@@ -76457,7 +76457,7 @@
         <v>2E-3</v>
       </c>
     </row>
-    <row r="23" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A23" s="39" t="s">
         <v>27</v>
       </c>
@@ -76627,7 +76627,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="24" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A24" s="39" t="s">
         <v>140</v>
       </c>
@@ -76797,7 +76797,7 @@
         <v>4.2000000000000003E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A25" s="39" t="s">
         <v>124</v>
       </c>
@@ -76967,7 +76967,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="26" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A26" s="39" t="s">
         <v>33</v>
       </c>
@@ -77137,7 +77137,7 @@
         <v>9.7000000000000003E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A27" s="39" t="s">
         <v>330</v>
       </c>
@@ -77307,7 +77307,7 @@
         <v>0.218</v>
       </c>
     </row>
-    <row r="28" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A28" s="39" t="s">
         <v>134</v>
       </c>
@@ -77477,7 +77477,7 @@
         <v>0.23100000000000001</v>
       </c>
     </row>
-    <row r="29" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A29" s="39" t="s">
         <v>97</v>
       </c>
@@ -77647,7 +77647,7 @@
         <v>5.8999999999999997E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A30" s="39" t="s">
         <v>101</v>
       </c>
@@ -77817,7 +77817,7 @@
         <v>0.14699999999999999</v>
       </c>
     </row>
-    <row r="31" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A31" s="39" t="s">
         <v>230</v>
       </c>
@@ -77987,7 +77987,7 @@
         <v>0.16200000000000001</v>
       </c>
     </row>
-    <row r="32" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A32" s="39" t="s">
         <v>318</v>
       </c>
@@ -78157,7 +78157,7 @@
         <v>0.182</v>
       </c>
     </row>
-    <row r="33" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A33" s="39" t="s">
         <v>206</v>
       </c>
@@ -78327,7 +78327,7 @@
         <v>0.186</v>
       </c>
     </row>
-    <row r="34" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A34" s="39" t="s">
         <v>95</v>
       </c>
@@ -78497,7 +78497,7 @@
         <v>8.8999999999999996E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A35" s="39" t="s">
         <v>312</v>
       </c>
@@ -78667,7 +78667,7 @@
         <v>3.2000000000000001E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A36" s="39" t="s">
         <v>248</v>
       </c>
@@ -78837,7 +78837,7 @@
         <v>0.41099999999999998</v>
       </c>
     </row>
-    <row r="37" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A37" s="39" t="s">
         <v>232</v>
       </c>
@@ -79007,7 +79007,7 @@
         <v>0.435</v>
       </c>
     </row>
-    <row r="38" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A38" s="39" t="s">
         <v>118</v>
       </c>
@@ -79177,7 +79177,7 @@
         <v>0.109</v>
       </c>
     </row>
-    <row r="39" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A39" s="39" t="s">
         <v>194</v>
       </c>
@@ -79347,7 +79347,7 @@
         <v>0.23</v>
       </c>
     </row>
-    <row r="40" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A40" s="39" t="s">
         <v>156</v>
       </c>
@@ -79517,7 +79517,7 @@
         <v>0.21299999999999999</v>
       </c>
     </row>
-    <row r="41" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="41" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A41" s="39" t="s">
         <v>334</v>
       </c>
@@ -79687,7 +79687,7 @@
         <v>0.22700000000000001</v>
       </c>
     </row>
-    <row r="42" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="42" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A42" s="39" t="s">
         <v>43</v>
       </c>
@@ -79857,7 +79857,7 @@
         <v>0.22700000000000001</v>
       </c>
     </row>
-    <row r="43" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A43" s="39" t="s">
         <v>372</v>
       </c>
@@ -80027,7 +80027,7 @@
         <v>0.127</v>
       </c>
     </row>
-    <row r="44" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="44" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A44" s="39" t="s">
         <v>180</v>
       </c>
@@ -80197,7 +80197,7 @@
         <v>0.09</v>
       </c>
     </row>
-    <row r="45" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="45" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A45" s="39" t="s">
         <v>274</v>
       </c>
@@ -80367,7 +80367,7 @@
         <v>0.32700000000000001</v>
       </c>
     </row>
-    <row r="46" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="46" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A46" s="39" t="s">
         <v>49</v>
       </c>
@@ -80537,7 +80537,7 @@
         <v>0.16500000000000001</v>
       </c>
     </row>
-    <row r="47" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="47" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A47" s="39" t="s">
         <v>130</v>
       </c>
@@ -80707,7 +80707,7 @@
         <v>0.19900000000000001</v>
       </c>
     </row>
-    <row r="48" spans="1:56" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="48" spans="1:56" ht="20.100000000000001" customHeight="1">
       <c r="A48" s="39"/>
     </row>
   </sheetData>

</xml_diff>